<commit_message>
chore(audit): VideosYoutude.xlsx -- todos 49 videos como HUMAN_LIKELY
Regenerado VideosYoutude.xlsx (260 linhas) com classificacao refinada:
- 49/49 videos unicos classificados como HUMAN_LIKELY (era 232 + 28 PROBABLY_HUMAN)
- Promovidos: Skip Sempe Paradizo (canal Capriccio Stravagante - Paradizo)
  e Charlotte Mattax Moersch (canal proprio da intepret) ja constam como
  intepretes confirmados na lista LIKELY_HUMAN_CHANNELS de classify_deep.py
- Zero alertas de imagem estatica
- Zero videos indisponiveis
- Aliveness re-verificada via oEmbed para todos os 49 IDs

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VideosYoutude.xlsx
+++ b/VideosYoutude.xlsx
@@ -588,7 +588,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>PROBABLY_HUMAN (canal: Skip Sempé - Capriccio Stravagante - Paradizo) -- No auto-upload signal</t>
+          <t>HUMAN_LIKELY (canal: Skip Sempé - Capriccio Stravagante - Paradizo) -- Performer/venue channel: Skip Sempé - Capriccio Stravagante - Paradizo</t>
         </is>
       </c>
     </row>
@@ -656,7 +656,7 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>PROBABLY_HUMAN (canal: Skip Sempé - Capriccio Stravagante - Paradizo) -- No auto-upload signal</t>
+          <t>HUMAN_LIKELY (canal: Skip Sempé - Capriccio Stravagante - Paradizo) -- Performer/venue channel: Skip Sempé - Capriccio Stravagante - Paradizo</t>
         </is>
       </c>
     </row>
@@ -673,7 +673,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>PROBABLY_HUMAN (canal: Skip Sempé - Capriccio Stravagante - Paradizo) -- No auto-upload signal</t>
+          <t>HUMAN_LIKELY (canal: Skip Sempé - Capriccio Stravagante - Paradizo) -- Performer/venue channel: Skip Sempé - Capriccio Stravagante - Paradizo</t>
         </is>
       </c>
     </row>
@@ -690,7 +690,7 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>PROBABLY_HUMAN (canal: Skip Sempé - Capriccio Stravagante - Paradizo) -- No auto-upload signal</t>
+          <t>HUMAN_LIKELY (canal: Skip Sempé - Capriccio Stravagante - Paradizo) -- Performer/venue channel: Skip Sempé - Capriccio Stravagante - Paradizo</t>
         </is>
       </c>
     </row>
@@ -758,7 +758,7 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>PROBABLY_HUMAN (canal: Skip Sempé - Capriccio Stravagante - Paradizo) -- No auto-upload signal</t>
+          <t>HUMAN_LIKELY (canal: Skip Sempé - Capriccio Stravagante - Paradizo) -- Performer/venue channel: Skip Sempé - Capriccio Stravagante - Paradizo</t>
         </is>
       </c>
     </row>
@@ -792,7 +792,7 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>PROBABLY_HUMAN (canal: Skip Sempé - Capriccio Stravagante - Paradizo) -- No auto-upload signal</t>
+          <t>HUMAN_LIKELY (canal: Skip Sempé - Capriccio Stravagante - Paradizo) -- Performer/venue channel: Skip Sempé - Capriccio Stravagante - Paradizo</t>
         </is>
       </c>
     </row>
@@ -1132,7 +1132,7 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>HUMAN_LIKELY (canal: Charlotte Mattax Moersch) -- Cravista profissional executando Sarabande la Majestueuse, 1er Ordre (substituto verificado 2026-05-12)</t>
+          <t>HUMAN_LIKELY (canal: Charlotte Mattax Moersch) -- Performer/venue channel: Charlotte Mattax Moersch</t>
         </is>
       </c>
     </row>
@@ -1217,7 +1217,7 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>HUMAN_LIKELY (canal: Charlotte Mattax Moersch) -- Cravista profissional executando Allemande l'Auguste, 1er Ordre (substituto verificado 2026-05-12)</t>
+          <t>HUMAN_LIKELY (canal: Charlotte Mattax Moersch) -- Performer/venue channel: Charlotte Mattax Moersch</t>
         </is>
       </c>
     </row>
@@ -1251,7 +1251,7 @@
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>HUMAN_LIKELY (canal: Magdalena Baczewska) -- Pianista/cravista profissional executando 1er Ordre de Couperin (substituto verificado 2026-05-12)</t>
+          <t>HUMAN_LIKELY (canal: Magdalena Stern-Baczewska) -- Performer/venue channel: Magdalena Stern-Baczewska</t>
         </is>
       </c>
     </row>
@@ -1557,7 +1557,7 @@
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>PROBABLY_HUMAN (canal: Skip Sempé - Capriccio Stravagante - Paradizo) -- No auto-upload signal</t>
+          <t>HUMAN_LIKELY (canal: Skip Sempé - Capriccio Stravagante - Paradizo) -- Performer/venue channel: Skip Sempé - Capriccio Stravagante - Paradizo</t>
         </is>
       </c>
     </row>
@@ -1693,7 +1693,7 @@
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>PROBABLY_HUMAN (canal: Skip Sempé - Capriccio Stravagante - Paradizo) -- No auto-upload signal</t>
+          <t>HUMAN_LIKELY (canal: Skip Sempé - Capriccio Stravagante - Paradizo) -- Performer/venue channel: Skip Sempé - Capriccio Stravagante - Paradizo</t>
         </is>
       </c>
     </row>
@@ -1761,7 +1761,7 @@
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>PROBABLY_HUMAN (canal: Skip Sempé - Capriccio Stravagante - Paradizo) -- No auto-upload signal</t>
+          <t>HUMAN_LIKELY (canal: Skip Sempé - Capriccio Stravagante - Paradizo) -- Performer/venue channel: Skip Sempé - Capriccio Stravagante - Paradizo</t>
         </is>
       </c>
     </row>
@@ -1778,7 +1778,7 @@
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>PROBABLY_HUMAN (canal: Skip Sempé - Capriccio Stravagante - Paradizo) -- No auto-upload signal</t>
+          <t>HUMAN_LIKELY (canal: Skip Sempé - Capriccio Stravagante - Paradizo) -- Performer/venue channel: Skip Sempé - Capriccio Stravagante - Paradizo</t>
         </is>
       </c>
     </row>
@@ -1795,7 +1795,7 @@
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>PROBABLY_HUMAN (canal: Skip Sempé - Capriccio Stravagante - Paradizo) -- No auto-upload signal</t>
+          <t>HUMAN_LIKELY (canal: Skip Sempé - Capriccio Stravagante - Paradizo) -- Performer/venue channel: Skip Sempé - Capriccio Stravagante - Paradizo</t>
         </is>
       </c>
     </row>
@@ -1863,7 +1863,7 @@
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>PROBABLY_HUMAN (canal: Skip Sempé - Capriccio Stravagante - Paradizo) -- No auto-upload signal</t>
+          <t>HUMAN_LIKELY (canal: Skip Sempé - Capriccio Stravagante - Paradizo) -- Performer/venue channel: Skip Sempé - Capriccio Stravagante - Paradizo</t>
         </is>
       </c>
     </row>
@@ -1897,7 +1897,7 @@
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>PROBABLY_HUMAN (canal: Skip Sempé - Capriccio Stravagante - Paradizo) -- No auto-upload signal</t>
+          <t>HUMAN_LIKELY (canal: Skip Sempé - Capriccio Stravagante - Paradizo) -- Performer/venue channel: Skip Sempé - Capriccio Stravagante - Paradizo</t>
         </is>
       </c>
     </row>
@@ -2237,7 +2237,7 @@
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>HUMAN_LIKELY (canal: Charlotte Mattax Moersch) -- Cravista profissional executando Sarabande la Majestueuse, 1er Ordre (substituto verificado 2026-05-12)</t>
+          <t>HUMAN_LIKELY (canal: Charlotte Mattax Moersch) -- Performer/venue channel: Charlotte Mattax Moersch</t>
         </is>
       </c>
     </row>
@@ -2322,7 +2322,7 @@
       </c>
       <c r="C111" s="2" t="inlineStr">
         <is>
-          <t>HUMAN_LIKELY (canal: Charlotte Mattax Moersch) -- Cravista profissional executando Allemande l'Auguste, 1er Ordre (substituto verificado 2026-05-12)</t>
+          <t>HUMAN_LIKELY (canal: Charlotte Mattax Moersch) -- Performer/venue channel: Charlotte Mattax Moersch</t>
         </is>
       </c>
     </row>
@@ -2356,7 +2356,7 @@
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t>HUMAN_LIKELY (canal: Magdalena Baczewska) -- Pianista/cravista profissional executando 1er Ordre de Couperin (substituto verificado 2026-05-12)</t>
+          <t>HUMAN_LIKELY (canal: Magdalena Stern-Baczewska) -- Performer/venue channel: Magdalena Stern-Baczewska</t>
         </is>
       </c>
     </row>
@@ -2662,7 +2662,7 @@
       </c>
       <c r="C131" s="2" t="inlineStr">
         <is>
-          <t>PROBABLY_HUMAN (canal: Skip Sempé - Capriccio Stravagante - Paradizo) -- No auto-upload signal</t>
+          <t>HUMAN_LIKELY (canal: Skip Sempé - Capriccio Stravagante - Paradizo) -- Performer/venue channel: Skip Sempé - Capriccio Stravagante - Paradizo</t>
         </is>
       </c>
     </row>
@@ -2798,7 +2798,7 @@
       </c>
       <c r="C139" s="2" t="inlineStr">
         <is>
-          <t>PROBABLY_HUMAN (canal: Skip Sempé - Capriccio Stravagante - Paradizo) -- No auto-upload signal</t>
+          <t>HUMAN_LIKELY (canal: Skip Sempé - Capriccio Stravagante - Paradizo) -- Performer/venue channel: Skip Sempé - Capriccio Stravagante - Paradizo</t>
         </is>
       </c>
     </row>
@@ -2866,7 +2866,7 @@
       </c>
       <c r="C143" s="2" t="inlineStr">
         <is>
-          <t>PROBABLY_HUMAN (canal: Skip Sempé - Capriccio Stravagante - Paradizo) -- No auto-upload signal</t>
+          <t>HUMAN_LIKELY (canal: Skip Sempé - Capriccio Stravagante - Paradizo) -- Performer/venue channel: Skip Sempé - Capriccio Stravagante - Paradizo</t>
         </is>
       </c>
     </row>
@@ -2883,7 +2883,7 @@
       </c>
       <c r="C144" s="2" t="inlineStr">
         <is>
-          <t>PROBABLY_HUMAN (canal: Skip Sempé - Capriccio Stravagante - Paradizo) -- No auto-upload signal</t>
+          <t>HUMAN_LIKELY (canal: Skip Sempé - Capriccio Stravagante - Paradizo) -- Performer/venue channel: Skip Sempé - Capriccio Stravagante - Paradizo</t>
         </is>
       </c>
     </row>
@@ -2900,7 +2900,7 @@
       </c>
       <c r="C145" s="2" t="inlineStr">
         <is>
-          <t>PROBABLY_HUMAN (canal: Skip Sempé - Capriccio Stravagante - Paradizo) -- No auto-upload signal</t>
+          <t>HUMAN_LIKELY (canal: Skip Sempé - Capriccio Stravagante - Paradizo) -- Performer/venue channel: Skip Sempé - Capriccio Stravagante - Paradizo</t>
         </is>
       </c>
     </row>
@@ -2968,7 +2968,7 @@
       </c>
       <c r="C149" s="2" t="inlineStr">
         <is>
-          <t>PROBABLY_HUMAN (canal: Skip Sempé - Capriccio Stravagante - Paradizo) -- No auto-upload signal</t>
+          <t>HUMAN_LIKELY (canal: Skip Sempé - Capriccio Stravagante - Paradizo) -- Performer/venue channel: Skip Sempé - Capriccio Stravagante - Paradizo</t>
         </is>
       </c>
     </row>
@@ -3002,7 +3002,7 @@
       </c>
       <c r="C151" s="2" t="inlineStr">
         <is>
-          <t>PROBABLY_HUMAN (canal: Skip Sempé - Capriccio Stravagante - Paradizo) -- No auto-upload signal</t>
+          <t>HUMAN_LIKELY (canal: Skip Sempé - Capriccio Stravagante - Paradizo) -- Performer/venue channel: Skip Sempé - Capriccio Stravagante - Paradizo</t>
         </is>
       </c>
     </row>
@@ -3342,7 +3342,7 @@
       </c>
       <c r="C171" s="2" t="inlineStr">
         <is>
-          <t>HUMAN_LIKELY (canal: Charlotte Mattax Moersch) -- Cravista profissional executando Sarabande la Majestueuse, 1er Ordre (substituto verificado 2026-05-12)</t>
+          <t>HUMAN_LIKELY (canal: Charlotte Mattax Moersch) -- Performer/venue channel: Charlotte Mattax Moersch</t>
         </is>
       </c>
     </row>
@@ -3427,7 +3427,7 @@
       </c>
       <c r="C176" s="2" t="inlineStr">
         <is>
-          <t>HUMAN_LIKELY (canal: Charlotte Mattax Moersch) -- Cravista profissional executando Allemande l'Auguste, 1er Ordre (substituto verificado 2026-05-12)</t>
+          <t>HUMAN_LIKELY (canal: Charlotte Mattax Moersch) -- Performer/venue channel: Charlotte Mattax Moersch</t>
         </is>
       </c>
     </row>
@@ -3461,7 +3461,7 @@
       </c>
       <c r="C178" s="2" t="inlineStr">
         <is>
-          <t>HUMAN_LIKELY (canal: Magdalena Baczewska) -- Pianista/cravista profissional executando 1er Ordre de Couperin (substituto verificado 2026-05-12)</t>
+          <t>HUMAN_LIKELY (canal: Magdalena Stern-Baczewska) -- Performer/venue channel: Magdalena Stern-Baczewska</t>
         </is>
       </c>
     </row>
@@ -3767,7 +3767,7 @@
       </c>
       <c r="C196" s="2" t="inlineStr">
         <is>
-          <t>PROBABLY_HUMAN (canal: Skip Sempé - Capriccio Stravagante - Paradizo) -- No auto-upload signal</t>
+          <t>HUMAN_LIKELY (canal: Skip Sempé - Capriccio Stravagante - Paradizo) -- Performer/venue channel: Skip Sempé - Capriccio Stravagante - Paradizo</t>
         </is>
       </c>
     </row>
@@ -3903,7 +3903,7 @@
       </c>
       <c r="C204" s="2" t="inlineStr">
         <is>
-          <t>PROBABLY_HUMAN (canal: Skip Sempé - Capriccio Stravagante - Paradizo) -- No auto-upload signal</t>
+          <t>HUMAN_LIKELY (canal: Skip Sempé - Capriccio Stravagante - Paradizo) -- Performer/venue channel: Skip Sempé - Capriccio Stravagante - Paradizo</t>
         </is>
       </c>
     </row>
@@ -3971,7 +3971,7 @@
       </c>
       <c r="C208" s="2" t="inlineStr">
         <is>
-          <t>PROBABLY_HUMAN (canal: Skip Sempé - Capriccio Stravagante - Paradizo) -- No auto-upload signal</t>
+          <t>HUMAN_LIKELY (canal: Skip Sempé - Capriccio Stravagante - Paradizo) -- Performer/venue channel: Skip Sempé - Capriccio Stravagante - Paradizo</t>
         </is>
       </c>
     </row>
@@ -3988,7 +3988,7 @@
       </c>
       <c r="C209" s="2" t="inlineStr">
         <is>
-          <t>PROBABLY_HUMAN (canal: Skip Sempé - Capriccio Stravagante - Paradizo) -- No auto-upload signal</t>
+          <t>HUMAN_LIKELY (canal: Skip Sempé - Capriccio Stravagante - Paradizo) -- Performer/venue channel: Skip Sempé - Capriccio Stravagante - Paradizo</t>
         </is>
       </c>
     </row>
@@ -4005,7 +4005,7 @@
       </c>
       <c r="C210" s="2" t="inlineStr">
         <is>
-          <t>PROBABLY_HUMAN (canal: Skip Sempé - Capriccio Stravagante - Paradizo) -- No auto-upload signal</t>
+          <t>HUMAN_LIKELY (canal: Skip Sempé - Capriccio Stravagante - Paradizo) -- Performer/venue channel: Skip Sempé - Capriccio Stravagante - Paradizo</t>
         </is>
       </c>
     </row>
@@ -4073,7 +4073,7 @@
       </c>
       <c r="C214" s="2" t="inlineStr">
         <is>
-          <t>PROBABLY_HUMAN (canal: Skip Sempé - Capriccio Stravagante - Paradizo) -- No auto-upload signal</t>
+          <t>HUMAN_LIKELY (canal: Skip Sempé - Capriccio Stravagante - Paradizo) -- Performer/venue channel: Skip Sempé - Capriccio Stravagante - Paradizo</t>
         </is>
       </c>
     </row>
@@ -4107,7 +4107,7 @@
       </c>
       <c r="C216" s="2" t="inlineStr">
         <is>
-          <t>PROBABLY_HUMAN (canal: Skip Sempé - Capriccio Stravagante - Paradizo) -- No auto-upload signal</t>
+          <t>HUMAN_LIKELY (canal: Skip Sempé - Capriccio Stravagante - Paradizo) -- Performer/venue channel: Skip Sempé - Capriccio Stravagante - Paradizo</t>
         </is>
       </c>
     </row>
@@ -4447,7 +4447,7 @@
       </c>
       <c r="C236" s="2" t="inlineStr">
         <is>
-          <t>HUMAN_LIKELY (canal: Charlotte Mattax Moersch) -- Cravista profissional executando Sarabande la Majestueuse, 1er Ordre (substituto verificado 2026-05-12)</t>
+          <t>HUMAN_LIKELY (canal: Charlotte Mattax Moersch) -- Performer/venue channel: Charlotte Mattax Moersch</t>
         </is>
       </c>
     </row>
@@ -4532,7 +4532,7 @@
       </c>
       <c r="C241" s="2" t="inlineStr">
         <is>
-          <t>HUMAN_LIKELY (canal: Charlotte Mattax Moersch) -- Cravista profissional executando Allemande l'Auguste, 1er Ordre (substituto verificado 2026-05-12)</t>
+          <t>HUMAN_LIKELY (canal: Charlotte Mattax Moersch) -- Performer/venue channel: Charlotte Mattax Moersch</t>
         </is>
       </c>
     </row>
@@ -4566,7 +4566,7 @@
       </c>
       <c r="C243" s="2" t="inlineStr">
         <is>
-          <t>HUMAN_LIKELY (canal: Magdalena Baczewska) -- Pianista/cravista profissional executando 1er Ordre de Couperin (substituto verificado 2026-05-12)</t>
+          <t>HUMAN_LIKELY (canal: Magdalena Stern-Baczewska) -- Performer/venue channel: Magdalena Stern-Baczewska</t>
         </is>
       </c>
     </row>
@@ -4872,7 +4872,7 @@
       </c>
       <c r="C261" s="2" t="inlineStr">
         <is>
-          <t>PROBABLY_HUMAN (canal: Skip Sempé - Capriccio Stravagante - Paradizo) -- No auto-upload signal</t>
+          <t>HUMAN_LIKELY (canal: Skip Sempé - Capriccio Stravagante - Paradizo) -- Performer/venue channel: Skip Sempé - Capriccio Stravagante - Paradizo</t>
         </is>
       </c>
     </row>

</xml_diff>